<commit_message>
격벽 P1 개구부 보강 M1 · M2 · M3 — srebar code 1 고정 길이(len)
- srebar code 1 의 8 번 칸 len : 적으면 ±len/2 고정 길이 (덕트가 밀고 개구부가 자르는 것은 같다)
- M1 세로 · M2 가로(−3 %) · M3 사선, 셋씩 · 간격 100 · 8-244 녹색 선에서 잰 자리
- 철근망(len 없음)의 결과는 그대로

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pxd9b9G4a1bcy9FpZN9nhs
</commit_message>
<xml_diff>
--- a/PSCBOX_BUKSIL_DIAPHRAGM_P1.xlsx
+++ b/PSCBOX_BUKSIL_DIAPHRAGM_P1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N219"/>
+  <dimension ref="A1:N236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3727,7 +3727,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t># ---- 다음에 넣을 것 : 가로 철근망 · 개구부 보강 (srebar code 1) — 세로 철근망은 맨 아래에 넣었다 ----</t>
+          <t># ---- 도면 메모 (8-244) : 면 철근 · 개구부 보강 — 철근 행은 맨 아래에 있다 ----</t>
         </is>
       </c>
     </row>
@@ -4037,6 +4037,365 @@
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t># ---- srebar code 1 : 개구부 보강 M1 · M2 · M3 (2026-10-18) — 길이 고정 (8 번 칸 len) ----</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t># srebar | id | code | dia | init x,y,rot | range | num | ctc | len | | | | z</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>#   len 을 적으면 길이가 고정이다 — 자리를 한가운데로 ±len/2. 외곽 피복이 줄이지 않고, 덕트가 밀고 개구부가 자르는 것은 철근망과 같다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>#   자리는 8-244 녹색 선 33 개(외곽선 쌍은 한 철근으로)에서 잼 — init 은 가운데 철근의 중점, 열차 간격은 도면 99 ~ 101.6 → 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>#     M1 H25 L 2,000 세로 : x ∓924 · ∓825 · ∓726 (왼쪽) / 725 · 824 · 925 (오른쪽) · 첫 줄이 개구부 옆면에서 126</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>#     M2 H25 L 2,000 가로 (−3 %) : 위 −4,487 · −4,587 · −4,687 / 아래 −6,424 · −6,525 · −6,624 (중심선 깊이)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>#     M3 H25 L 1,500 사선 : 모서리 접기 넷에 셋씩 · 도면 각 44.15° / 134.15°</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>#   ! 자리를 도면에서 가져왔으므로 도면과 맞는 것은 검증이 아니다 (중점 2.2 mm 안 · 길이 2 mm 안)</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>M1-L</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>1</v>
+      </c>
+      <c r="D228" t="n">
+        <v>25</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>-824.7,-5556,90</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>3</v>
+      </c>
+      <c r="H228" t="n">
+        <v>100</v>
+      </c>
+      <c r="I228" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>opening bar M1, vertical, left of the opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>M1-R</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>1</v>
+      </c>
+      <c r="D229" t="n">
+        <v>25</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>823.6,-5567.4,90</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>3</v>
+      </c>
+      <c r="H229" t="n">
+        <v>100</v>
+      </c>
+      <c r="I229" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>opening bar M1, vertical, right</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>M2-T</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>1</v>
+      </c>
+      <c r="D230" t="n">
+        <v>25</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>7.1,-4587,-1.7184</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>3</v>
+      </c>
+      <c r="H230" t="n">
+        <v>100</v>
+      </c>
+      <c r="I230" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>opening bar M2, above the opening (parallel to the -3% faces)</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>M2-B</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>1</v>
+      </c>
+      <c r="D231" t="n">
+        <v>25</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>-5.7,-6524.9,-1.7184</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>3</v>
+      </c>
+      <c r="H231" t="n">
+        <v>100</v>
+      </c>
+      <c r="I231" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>opening bar M2, below the opening</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>M3-UL</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>1</v>
+      </c>
+      <c r="D232" t="n">
+        <v>25</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>-614,-4766.1,44.15</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>3</v>
+      </c>
+      <c r="H232" t="n">
+        <v>100</v>
+      </c>
+      <c r="I232" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>opening bar M3, diagonal, upper-left chamfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>M3-UR</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>1</v>
+      </c>
+      <c r="D233" t="n">
+        <v>25</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>636.9,-4782.6,134.15</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>3</v>
+      </c>
+      <c r="H233" t="n">
+        <v>100</v>
+      </c>
+      <c r="I233" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>opening bar M3, diagonal, upper-right chamfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>M3-LL</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>1</v>
+      </c>
+      <c r="D234" t="n">
+        <v>25</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>-627.3,-6307.7,134.15</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>3</v>
+      </c>
+      <c r="H234" t="n">
+        <v>100</v>
+      </c>
+      <c r="I234" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>opening bar M3, diagonal, lower-left chamfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>srebar</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>M3-LR</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>1</v>
+      </c>
+      <c r="D235" t="n">
+        <v>25</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>622.3,-6342,44.15</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>3</v>
+      </c>
+      <c r="H235" t="n">
+        <v>100</v>
+      </c>
+      <c r="I235" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>opening bar M3, diagonal, lower-right chamfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
         <is>
           <t>end</t>
         </is>

</xml_diff>